<commit_message>
Updated project files and removed unwanted files
</commit_message>
<xml_diff>
--- a/Dashboard/FRESHMART/FRESHMART DASHBOARD.xlsx
+++ b/Dashboard/FRESHMART/FRESHMART DASHBOARD.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5eb3c2e9862f82c0/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Subha\02_Excel\Project\Dashboard\FRESHMART\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67B02476-9324-4CDE-92CE-591E01CA0C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE2DBEF-F981-4DB6-A9E1-B4B19DFCEB6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FRESHMART SALES DASHBOARD" sheetId="1" r:id="rId1"/>
@@ -312,10 +312,10 @@
     <numFmt numFmtId="164" formatCode="\₹\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="\₹\ #,##0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -633,7 +633,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -662,28 +662,55 @@
     <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -696,6 +723,11 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -705,16 +737,6 @@
     <xf numFmtId="3" fontId="6" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -742,44 +764,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2645,44 +2639,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -2709,14 +2703,32 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -2743,6 +2755,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -2754,166 +2784,162 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
+            <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
@@ -2923,404 +2949,409 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:T100"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="20" width="12" customWidth="1"/>
     <col min="21" max="22" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="31" t="s">
+    <row r="1" spans="2:20" ht="24" customHeight="1"/>
+    <row r="2" spans="2:20" ht="24" customHeight="1">
+      <c r="B2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
-      <c r="S2" s="32"/>
-      <c r="T2" s="33"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
+      <c r="P2" s="20"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="20"/>
+      <c r="S2" s="20"/>
+      <c r="T2" s="21"/>
     </row>
-    <row r="3" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="34"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
-      <c r="S3" s="15"/>
-      <c r="T3" s="35"/>
+    <row r="3" spans="2:20" ht="24" customHeight="1">
+      <c r="B3" s="22"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="24"/>
     </row>
-    <row r="4" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="37"/>
-      <c r="K4" s="37"/>
-      <c r="L4" s="37"/>
-      <c r="M4" s="37"/>
-      <c r="N4" s="37"/>
-      <c r="O4" s="37"/>
-      <c r="P4" s="37"/>
-      <c r="Q4" s="37"/>
-      <c r="R4" s="37"/>
-      <c r="S4" s="37"/>
-      <c r="T4" s="38"/>
+    <row r="4" spans="2:20" ht="24" customHeight="1">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+      <c r="R4" s="26"/>
+      <c r="S4" s="26"/>
+      <c r="T4" s="27"/>
     </row>
-    <row r="5" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="10" t="s">
+    <row r="5" spans="2:20" ht="24" customHeight="1"/>
+    <row r="6" spans="2:20" ht="24" customHeight="1">
+      <c r="B6" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="27" t="s">
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="28" t="s">
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="24" t="s">
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="23" t="s">
+      <c r="O6" s="30"/>
+      <c r="P6" s="30"/>
+      <c r="Q6" s="31"/>
+      <c r="R6" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="S6" s="13"/>
-      <c r="T6" s="14"/>
+      <c r="S6" s="30"/>
+      <c r="T6" s="31"/>
     </row>
-    <row r="7" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="48" t="s">
+    <row r="7" spans="2:20" ht="24" customHeight="1">
+      <c r="B7" s="57" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="17"/>
-      <c r="T7" s="18"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="34"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="33"/>
+      <c r="Q7" s="34"/>
+      <c r="R7" s="32"/>
+      <c r="S7" s="33"/>
+      <c r="T7" s="34"/>
     </row>
-    <row r="8" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="51"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="25">
+    <row r="8" spans="2:20" ht="24" customHeight="1">
+      <c r="B8" s="58"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="36">
         <f>Calculations!E2</f>
         <v>12948632.6</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="26">
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="37">
         <f>Calculations!E3</f>
         <v>2037319.89</v>
       </c>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="30">
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="44">
         <f>Calculations!E4</f>
         <v>8323</v>
       </c>
-      <c r="O8" s="13"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="29">
+      <c r="O8" s="30"/>
+      <c r="P8" s="30"/>
+      <c r="Q8" s="31"/>
+      <c r="R8" s="43">
         <f>Calculations!E5</f>
         <v>2490</v>
       </c>
-      <c r="S8" s="13"/>
-      <c r="T8" s="14"/>
+      <c r="S8" s="30"/>
+      <c r="T8" s="31"/>
     </row>
-    <row r="9" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="54"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="56"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="18"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="17"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="16"/>
-      <c r="S9" s="17"/>
-      <c r="T9" s="18"/>
+    <row r="9" spans="2:20" ht="24" customHeight="1">
+      <c r="B9" s="32"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="33"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="33"/>
+      <c r="P9" s="33"/>
+      <c r="Q9" s="34"/>
+      <c r="R9" s="32"/>
+      <c r="S9" s="33"/>
+      <c r="T9" s="34"/>
     </row>
-    <row r="10" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="10" t="s">
+    <row r="10" spans="2:20" ht="24" customHeight="1"/>
+    <row r="11" spans="2:20" ht="24" customHeight="1">
+      <c r="B11" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="19" t="s">
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="19" t="s">
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="21"/>
-      <c r="P11" s="19" t="s">
+      <c r="L11" s="40"/>
+      <c r="M11" s="40"/>
+      <c r="N11" s="40"/>
+      <c r="O11" s="41"/>
+      <c r="P11" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="Q11" s="20"/>
-      <c r="R11" s="20"/>
-      <c r="S11" s="20"/>
-      <c r="T11" s="21"/>
+      <c r="Q11" s="40"/>
+      <c r="R11" s="40"/>
+      <c r="S11" s="40"/>
+      <c r="T11" s="41"/>
     </row>
-    <row r="12" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="57" t="s">
+    <row r="12" spans="2:20" ht="27.75" customHeight="1">
+      <c r="C12" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="D12" s="58"/>
-      <c r="E12" s="59"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="12"/>
     </row>
-    <row r="13" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="60"/>
-      <c r="C13" s="57" t="s">
+    <row r="13" spans="2:20" ht="27.75" customHeight="1">
+      <c r="B13" s="13"/>
+      <c r="C13" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D13" s="61"/>
-      <c r="E13" s="62"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="15"/>
     </row>
-    <row r="14" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="63"/>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
-      <c r="E14" s="65"/>
+    <row r="14" spans="2:20" ht="27.75" customHeight="1">
+      <c r="B14" s="16"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18"/>
     </row>
-    <row r="15" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="10" t="s">
+    <row r="15" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="16" spans="2:20" ht="27.75" customHeight="1">
+      <c r="B16" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="12"/>
+      <c r="C16" s="55"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="56"/>
     </row>
-    <row r="17" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="39" t="s">
+    <row r="17" spans="2:20" ht="27.75" customHeight="1">
+      <c r="B17" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="41"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="47"/>
     </row>
-    <row r="18" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="42"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="44"/>
+    <row r="18" spans="2:20" ht="27.75" customHeight="1">
+      <c r="B18" s="48"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
     </row>
-    <row r="19" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="45"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="47"/>
+    <row r="19" spans="2:20" ht="27.75" customHeight="1">
+      <c r="B19" s="51"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="53"/>
     </row>
-    <row r="20" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F21" s="19" t="s">
+    <row r="20" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="21" spans="2:20" ht="27.75" customHeight="1">
+      <c r="F21" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="19" t="s">
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="41"/>
+      <c r="K21" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="L21" s="20"/>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="21"/>
-      <c r="P21" s="19" t="s">
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="41"/>
+      <c r="P21" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="Q21" s="20"/>
-      <c r="R21" s="20"/>
-      <c r="S21" s="20"/>
-      <c r="T21" s="21"/>
+      <c r="Q21" s="40"/>
+      <c r="R21" s="40"/>
+      <c r="S21" s="40"/>
+      <c r="T21" s="41"/>
     </row>
-    <row r="22" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="2:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="34" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="6:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="6:20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="6:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F43" s="22"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="15"/>
-      <c r="J43" s="15"/>
-      <c r="K43" s="15"/>
-      <c r="L43" s="15"/>
-      <c r="M43" s="15"/>
-      <c r="N43" s="15"/>
-      <c r="O43" s="15"/>
-      <c r="P43" s="15"/>
-      <c r="Q43" s="15"/>
-      <c r="R43" s="15"/>
-      <c r="S43" s="15"/>
-      <c r="T43" s="15"/>
+    <row r="22" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="23" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="24" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="25" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="26" spans="2:20" ht="24" customHeight="1"/>
+    <row r="27" spans="2:20" ht="24" customHeight="1"/>
+    <row r="28" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="29" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="30" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="31" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="32" spans="2:20" ht="27.75" customHeight="1"/>
+    <row r="33" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="34" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="35" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="36" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="37" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="38" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="39" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="40" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="41" spans="6:20" ht="27.75" customHeight="1"/>
+    <row r="42" spans="6:20" ht="24" customHeight="1"/>
+    <row r="43" spans="6:20" ht="24" customHeight="1">
+      <c r="F43" s="28"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="23"/>
+      <c r="J43" s="23"/>
+      <c r="K43" s="23"/>
+      <c r="L43" s="23"/>
+      <c r="M43" s="23"/>
+      <c r="N43" s="23"/>
+      <c r="O43" s="23"/>
+      <c r="P43" s="23"/>
+      <c r="Q43" s="23"/>
+      <c r="R43" s="23"/>
+      <c r="S43" s="23"/>
+      <c r="T43" s="23"/>
     </row>
-    <row r="44" spans="6:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15"/>
-      <c r="I44" s="15"/>
-      <c r="J44" s="15"/>
-      <c r="K44" s="15"/>
-      <c r="L44" s="15"/>
-      <c r="M44" s="15"/>
-      <c r="N44" s="15"/>
-      <c r="O44" s="15"/>
-      <c r="P44" s="15"/>
-      <c r="Q44" s="15"/>
-      <c r="R44" s="15"/>
-      <c r="S44" s="15"/>
-      <c r="T44" s="15"/>
+    <row r="44" spans="6:20" ht="24" customHeight="1">
+      <c r="F44" s="23"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="23"/>
+      <c r="K44" s="23"/>
+      <c r="L44" s="23"/>
+      <c r="M44" s="23"/>
+      <c r="N44" s="23"/>
+      <c r="O44" s="23"/>
+      <c r="P44" s="23"/>
+      <c r="Q44" s="23"/>
+      <c r="R44" s="23"/>
+      <c r="S44" s="23"/>
+      <c r="T44" s="23"/>
     </row>
-    <row r="45" spans="6:20" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="6:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="6:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="6:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="6:20" ht="24" customHeight="1"/>
+    <row r="46" spans="6:20" ht="15.75" customHeight="1"/>
+    <row r="47" spans="6:20" ht="15.75" customHeight="1"/>
+    <row r="48" spans="6:20" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="51" ht="15.75" customHeight="1"/>
+    <row r="52" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1"/>
+    <row r="57" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="60" ht="15.75" customHeight="1"/>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1"/>
+    <row r="64" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="F21:J21"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B7:E9"/>
+    <mergeCell ref="B11:E11"/>
     <mergeCell ref="B2:T4"/>
     <mergeCell ref="F43:T44"/>
     <mergeCell ref="R6:T7"/>
@@ -3337,11 +3368,6 @@
     <mergeCell ref="P11:T11"/>
     <mergeCell ref="P21:T21"/>
     <mergeCell ref="K21:O21"/>
-    <mergeCell ref="F21:J21"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B7:E9"/>
-    <mergeCell ref="B11:E11"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="B17" xr:uid="{00000000-0002-0000-0000-000001000000}">
@@ -3354,21 +3380,21 @@
       <formula1>"All,Cash,Credit Card,Debit Card,EMI,Net Banking,UPI"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup paperSize="8" orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="39" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:W100"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="23" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -3425,7 +3451,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" ht="14.4">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
@@ -3482,7 +3508,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" ht="14.4">
       <c r="A3" s="2" t="s">
         <v>36</v>
       </c>
@@ -3539,7 +3565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" ht="14.4">
       <c r="A4" s="2" t="s">
         <v>44</v>
       </c>
@@ -3592,7 +3618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" ht="14.4">
       <c r="A5" s="2" t="s">
         <v>51</v>
       </c>
@@ -3641,7 +3667,7 @@
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
     </row>
-    <row r="6" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" ht="14.4">
       <c r="A6" s="2" t="s">
         <v>57</v>
       </c>
@@ -3686,7 +3712,7 @@
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
     </row>
-    <row r="7" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" ht="14.4">
       <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
@@ -3731,7 +3757,7 @@
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
     </row>
-    <row r="8" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" ht="14.4">
       <c r="A8" s="2" t="s">
         <v>67</v>
       </c>
@@ -3772,7 +3798,7 @@
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
     </row>
-    <row r="9" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" ht="14.4">
       <c r="A9" s="2" t="s">
         <v>71</v>
       </c>
@@ -3813,7 +3839,7 @@
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
     </row>
-    <row r="10" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="14.4">
       <c r="A10" s="2" t="s">
         <v>75</v>
       </c>
@@ -3850,7 +3876,7 @@
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
     </row>
-    <row r="11" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="14.4">
       <c r="A11" s="2" t="s">
         <v>78</v>
       </c>
@@ -3887,7 +3913,7 @@
       <c r="V11" s="2"/>
       <c r="W11" s="2"/>
     </row>
-    <row r="12" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="14.4">
       <c r="A12" s="2" t="s">
         <v>81</v>
       </c>
@@ -3916,7 +3942,7 @@
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
     </row>
-    <row r="13" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="14.4">
       <c r="A13" s="2" t="s">
         <v>82</v>
       </c>
@@ -3945,86 +3971,86 @@
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" ht="15.75" customHeight="1"/>
+    <row r="22" ht="15.75" customHeight="1"/>
+    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1"/>
+    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="37" ht="15.75" customHeight="1"/>
+    <row r="38" ht="15.75" customHeight="1"/>
+    <row r="39" ht="15.75" customHeight="1"/>
+    <row r="40" ht="15.75" customHeight="1"/>
+    <row r="41" ht="15.75" customHeight="1"/>
+    <row r="42" ht="15.75" customHeight="1"/>
+    <row r="43" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1"/>
+    <row r="45" ht="15.75" customHeight="1"/>
+    <row r="46" ht="15.75" customHeight="1"/>
+    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="51" ht="15.75" customHeight="1"/>
+    <row r="52" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1"/>
+    <row r="57" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="60" ht="15.75" customHeight="1"/>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1"/>
+    <row r="64" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -4034,12 +4060,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:W100"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="23" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" ht="14.4">
       <c r="A1" s="6" t="s">
         <v>83</v>
       </c>
@@ -4094,7 +4120,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" ht="14.4">
       <c r="A2" s="6" t="s">
         <v>85</v>
       </c>
@@ -4163,7 +4189,7 @@
         <v>2821365</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" ht="14.4">
       <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
@@ -4232,7 +4258,7 @@
         <v>2065964</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" ht="14.4">
       <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
@@ -4295,7 +4321,7 @@
         <v>1858745</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" ht="14.4">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -4353,7 +4379,7 @@
         <v>1624891</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" ht="14.4">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -4406,7 +4432,7 @@
         <v>1247558</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" ht="14.4">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -4459,7 +4485,7 @@
         <v>932114</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" ht="14.4">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -4512,7 +4538,7 @@
         <v>712368</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" ht="14.4">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -4565,7 +4591,7 @@
         <v>561285</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="14.4">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -4612,7 +4638,7 @@
       <c r="V10" s="6"/>
       <c r="W10" s="6"/>
     </row>
-    <row r="11" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="14.4">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -4654,7 +4680,7 @@
       <c r="V11" s="6"/>
       <c r="W11" s="6"/>
     </row>
-    <row r="12" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="14.4">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -4684,7 +4710,7 @@
       <c r="V12" s="6"/>
       <c r="W12" s="6"/>
     </row>
-    <row r="13" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="14.4">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -4714,86 +4740,86 @@
       <c r="V13" s="6"/>
       <c r="W13" s="6"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" ht="15.75" customHeight="1"/>
+    <row r="22" ht="15.75" customHeight="1"/>
+    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1"/>
+    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="37" ht="15.75" customHeight="1"/>
+    <row r="38" ht="15.75" customHeight="1"/>
+    <row r="39" ht="15.75" customHeight="1"/>
+    <row r="40" ht="15.75" customHeight="1"/>
+    <row r="41" ht="15.75" customHeight="1"/>
+    <row r="42" ht="15.75" customHeight="1"/>
+    <row r="43" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1"/>
+    <row r="45" ht="15.75" customHeight="1"/>
+    <row r="46" ht="15.75" customHeight="1"/>
+    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="51" ht="15.75" customHeight="1"/>
+    <row r="52" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1"/>
+    <row r="57" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="60" ht="15.75" customHeight="1"/>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1"/>
+    <row r="64" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>